<commit_message>
Rater sheet: a full stop on every line without terminal punctuation, the same rule for both systems (protocol v2.26)
Four (c) lines changed; the XLSX is regenerated. Every line now ends with a full stop, starts with a
capital and has no stray spaces. One form difference stays: 3 (a) lines quote a phrase, no (c) line does.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/track_2b/results/native_check/rater/german_lines.xlsx
+++ b/track_2b/results/native_check/rater/german_lines.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="106">
   <si>
     <t xml:space="preserve">Native-speaker check: English → German</t>
   </si>
@@ -149,7 +149,7 @@
     <t xml:space="preserve">The Schengen zone, however, works somewhat like one country in this respect.</t>
   </si>
   <si>
-    <t xml:space="preserve">Der Schengen-Raum funktioniert in dieser Hinsicht ein wenig wie ein Land</t>
+    <t xml:space="preserve">Der Schengen-Raum funktioniert in dieser Hinsicht ein wenig wie ein Land.</t>
   </si>
   <si>
     <t xml:space="preserve">Bishkek was described as sinking into a state of "anarchy" by one observer, as gangs of people roamed the streets and plundered stores of consumer goods.</t>
@@ -308,9 +308,6 @@
     <t xml:space="preserve">Löwen sind die sozialen Katzen, die in großen Gruppen namens Rudeln leben.</t>
   </si>
   <si>
-    <t xml:space="preserve">Als Ergebnis rauchen die Darsteller auf der Bühne Cannabis-Joints, und das Theater selbst ermutigt das Publikum, mitzumachen</t>
-  </si>
-  <si>
     <t xml:space="preserve">A civilization is a singular culture shared by a significant large group of people who live and work co-operatively, a society.</t>
   </si>
   <si>
@@ -320,7 +317,7 @@
     <t xml:space="preserve">Es gibt natürlich christliche theologische Erklärungen für diese Tradition, aber es könnte durchaus ein vorchristliches Frühlings- und Fruchtbarkeitsritual sein.</t>
   </si>
   <si>
-    <t xml:space="preserve">Soziale Löwen leben in Rudeln zusammen und sind Katzen</t>
+    <t xml:space="preserve">Soziale Löwen leben in Rudeln zusammen und sind Katzen.</t>
   </si>
   <si>
     <t xml:space="preserve">Last week, METI announced that Apple had informed it of 34 additional overheating incidents, which the company called "non-serious."</t>
@@ -333,9 +330,6 @@
   </si>
   <si>
     <t xml:space="preserve">Letzte Woche meldete METI, Apple über 34 weitere Überhitzungsfälle, als nicht schwerwiegend eingestuft.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Eine Zivilisation ist eine einzigartige Kultur, die von einer großen Gruppe von Menschen geteilt wird, die kooperativ leben und arbeiten, eine Gesellschaft</t>
   </si>
   <si>
     <t xml:space="preserve">Dies ist eine wichtige Methode, um einige Verben von einigen Objekten zu unterscheiden.</t>
@@ -1243,7 +1237,7 @@
         <v>89</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="D38" s="3"/>
       <c r="E38" s="3"/>
@@ -1270,10 +1264,10 @@
         <v>39</v>
       </c>
       <c r="B40" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C40" s="2" t="s">
         <v>95</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>96</v>
       </c>
       <c r="D40" s="3"/>
       <c r="E40" s="3"/>
@@ -1303,7 +1297,7 @@
         <v>84</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D42" s="3"/>
       <c r="E42" s="3"/>
@@ -1318,7 +1312,7 @@
         <v>92</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D43" s="3"/>
       <c r="E43" s="3"/>
@@ -1330,10 +1324,10 @@
         <v>43</v>
       </c>
       <c r="B44" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C44" s="2" t="s">
         <v>99</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>100</v>
       </c>
       <c r="D44" s="3"/>
       <c r="E44" s="3"/>
@@ -1348,7 +1342,7 @@
         <v>48</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D45" s="3"/>
       <c r="E45" s="3"/>
@@ -1360,10 +1354,10 @@
         <v>45</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D46" s="3"/>
       <c r="E46" s="3"/>
@@ -1375,10 +1369,10 @@
         <v>46</v>
       </c>
       <c r="B47" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C47" s="2" t="s">
         <v>95</v>
-      </c>
-      <c r="C47" s="2" t="s">
-        <v>103</v>
       </c>
       <c r="D47" s="3"/>
       <c r="E47" s="3"/>
@@ -1393,7 +1387,7 @@
         <v>86</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D48" s="3"/>
       <c r="E48" s="3"/>
@@ -1408,7 +1402,7 @@
         <v>52</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D49" s="3"/>
       <c r="E49" s="3"/>
@@ -1423,7 +1417,7 @@
         <v>74</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D50" s="3"/>
       <c r="E50" s="3"/>
@@ -1438,7 +1432,7 @@
         <v>44</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D51" s="3"/>
       <c r="E51" s="3"/>

</xml_diff>